<commit_message>
Final project update: dataset + unit tests + clean structure
</commit_message>
<xml_diff>
--- a/scraping/loans/loan_data.xlsx
+++ b/scraping/loans/loan_data.xlsx
@@ -566,7 +566,7 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>2026-04-18 14:16:32</t>
+          <t>2026-04-18 14:57:01</t>
         </is>
       </c>
     </row>
@@ -624,7 +624,7 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>2026-04-18 14:16:32</t>
+          <t>2026-04-18 14:57:01</t>
         </is>
       </c>
     </row>
@@ -686,7 +686,7 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>2026-04-18 14:16:33</t>
+          <t>2026-04-18 14:57:03</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>2026-04-18 14:16:34</t>
+          <t>2026-04-18 14:57:04</t>
         </is>
       </c>
     </row>
@@ -804,7 +804,7 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>2026-04-18 14:16:35</t>
+          <t>2026-04-18 14:57:04</t>
         </is>
       </c>
     </row>

</xml_diff>